<commit_message>
Ajuste y precisión de visibilidad + Excel
</commit_message>
<xml_diff>
--- a/app/info/Matriz Criterios 1.xlsx
+++ b/app/info/Matriz Criterios 1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Desktop\Coding Project\PROYECTAMOS\Alcaldia\CodexDashboard\info\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Desktop\Coding Project\PROYECTAMOS\Alcaldia\REPOSITORIOS-AZURE\DDCS-back-reportes\app\info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE73D33-5A1C-4E07-895A-8031D82E3592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD577748-1614-4738-9A44-A96116486C51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="252">
   <si>
     <t>Dimensión</t>
   </si>
@@ -149,9 +149,6 @@
     <t>Base de datos de calificación de habilidades</t>
   </si>
   <si>
-    <t>Presencial Red CADE, Ferias</t>
-  </si>
-  <si>
     <t>Cumplimiento del protocolo de atención</t>
   </si>
   <si>
@@ -173,9 +170,6 @@
     <t>Tiempo total empleado</t>
   </si>
   <si>
-    <t>Presencial Ferias, Punto Propio, Red CADE</t>
-  </si>
-  <si>
     <t>1 - (Tiempo total empleado / Máximo de tiempo total empleado en el universo)</t>
   </si>
   <si>
@@ -795,6 +789,18 @@
   </si>
   <si>
     <t>Accesibilidad instalada en el punto de atención</t>
+  </si>
+  <si>
+    <t>Presencial Red CADE, Centros de encuentros</t>
+  </si>
+  <si>
+    <t>Presencial Ferias, Punto Propio</t>
+  </si>
+  <si>
+    <t>Presencial Centros de encuentros, Punto Propio, Alcaldías Locales</t>
+  </si>
+  <si>
+    <t>Presencial Ferias, Punto Propio, Alcaldías Locales</t>
   </si>
 </sst>
 </file>
@@ -1082,6 +1088,18 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1104,18 +1122,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1342,7 +1348,7 @@
   <dimension ref="A1:M958"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.59765625" style="30" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.59765625" style="21" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24" style="2" customWidth="1"/>
     <col min="3" max="3" width="33.796875" style="3" customWidth="1"/>
     <col min="4" max="4" width="29.69921875" style="2" customWidth="1"/>
@@ -1356,64 +1362,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="B1" s="23" t="s">
+      <c r="A1" s="22" t="s">
+        <v>206</v>
+      </c>
+      <c r="B1" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="25" t="s">
-        <v>147</v>
-      </c>
-      <c r="E1" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="F1" s="25" t="s">
+      <c r="D1" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="J1" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="G1" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="I1" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="J1" s="19" t="s">
+      <c r="L1" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="M1" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="K1" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="L1" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="M1" s="19" t="s">
-        <v>57</v>
-      </c>
     </row>
     <row r="2" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="20"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="24"/>
     </row>
     <row r="3" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
-        <v>209</v>
+      <c r="A3" s="19" t="s">
+        <v>207</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>6</v>
@@ -1423,36 +1429,36 @@
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F3" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K3" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>67</v>
       </c>
       <c r="L3" s="4" t="s">
         <v>4</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A4" s="29" t="s">
-        <v>210</v>
+      <c r="A4" s="20" t="s">
+        <v>208</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>6</v>
@@ -1462,36 +1468,36 @@
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J4" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="K4" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A5" s="28" t="s">
-        <v>211</v>
+      <c r="A5" s="19" t="s">
+        <v>209</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>7</v>
@@ -1504,19 +1510,19 @@
         <v>19</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>22</v>
@@ -1525,12 +1531,12 @@
         <v>4</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="45" x14ac:dyDescent="0.3">
-      <c r="A6" s="28" t="s">
-        <v>212</v>
+      <c r="A6" s="19" t="s">
+        <v>210</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>7</v>
@@ -1543,19 +1549,19 @@
         <v>20</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>22</v>
@@ -1564,12 +1570,12 @@
         <v>4</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="45" x14ac:dyDescent="0.3">
-      <c r="A7" s="28" t="s">
-        <v>213</v>
+      <c r="A7" s="19" t="s">
+        <v>211</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>7</v>
@@ -1582,19 +1588,19 @@
         <v>21</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G7" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="I7" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>86</v>
-      </c>
       <c r="J7" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>22</v>
@@ -1603,12 +1609,12 @@
         <v>4</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="60" x14ac:dyDescent="0.3">
-      <c r="A8" s="28" t="s">
-        <v>214</v>
+      <c r="A8" s="19" t="s">
+        <v>212</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>7</v>
@@ -1618,22 +1624,22 @@
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>22</v>
@@ -1642,12 +1648,12 @@
         <v>4</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="45" x14ac:dyDescent="0.3">
-      <c r="A9" s="28" t="s">
-        <v>215</v>
+      <c r="A9" s="19" t="s">
+        <v>213</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>7</v>
@@ -1660,19 +1666,19 @@
         <v>23</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K9" s="4" t="s">
         <v>22</v>
@@ -1681,37 +1687,37 @@
         <v>4</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:13" s="8" customFormat="1" ht="45" x14ac:dyDescent="0.3">
-      <c r="A10" s="28" t="s">
-        <v>216</v>
+      <c r="A10" s="19" t="s">
+        <v>214</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7" t="s">
         <v>10</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>22</v>
@@ -1720,37 +1726,37 @@
         <v>4</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="45" x14ac:dyDescent="0.3">
-      <c r="A11" s="28" t="s">
-        <v>217</v>
+      <c r="A11" s="19" t="s">
+        <v>215</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K11" s="4" t="s">
         <v>22</v>
@@ -1759,37 +1765,37 @@
         <v>4</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="45" x14ac:dyDescent="0.3">
-      <c r="A12" s="28" t="s">
-        <v>218</v>
+      <c r="A12" s="19" t="s">
+        <v>216</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
         <v>24</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>25</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K12" s="4" t="s">
         <v>22</v>
@@ -1798,37 +1804,37 @@
         <v>4</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="45" x14ac:dyDescent="0.3">
-      <c r="A13" s="28" t="s">
-        <v>219</v>
+      <c r="A13" s="19" t="s">
+        <v>217</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K13" s="4" t="s">
         <v>22</v>
@@ -1837,37 +1843,37 @@
         <v>4</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A14" s="28" t="s">
-        <v>220</v>
+      <c r="A14" s="19" t="s">
+        <v>218</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D14" s="4"/>
       <c r="E14" s="10" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I14" s="10">
         <v>240</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>22</v>
@@ -1876,37 +1882,37 @@
         <v>4</v>
       </c>
       <c r="M14" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A15" s="28" t="s">
-        <v>221</v>
+      <c r="A15" s="19" t="s">
+        <v>219</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="10" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I15" s="10">
         <v>240</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K15" s="4" t="s">
         <v>22</v>
@@ -1915,37 +1921,37 @@
         <v>4</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A16" s="28" t="s">
-        <v>222</v>
+      <c r="A16" s="19" t="s">
+        <v>220</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="10" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="I16" s="10">
         <v>240</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K16" s="4" t="s">
         <v>22</v>
@@ -1954,12 +1960,12 @@
         <v>4</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:13" s="8" customFormat="1" ht="165" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="29" t="s">
-        <v>223</v>
+      <c r="A17" s="20" t="s">
+        <v>221</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>12</v>
@@ -1971,22 +1977,22 @@
         <v>16</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K17" s="7" t="s">
         <v>31</v>
@@ -1995,12 +2001,12 @@
         <v>26</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="180" x14ac:dyDescent="0.3">
-      <c r="A18" s="29" t="s">
-        <v>224</v>
+      <c r="A18" s="20" t="s">
+        <v>222</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>12</v>
@@ -2012,22 +2018,22 @@
         <v>16</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K18" s="7" t="s">
         <v>31</v>
@@ -2036,12 +2042,12 @@
         <v>26</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A19" s="29" t="s">
-        <v>225</v>
+      <c r="A19" s="20" t="s">
+        <v>223</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>12</v>
@@ -2056,19 +2062,19 @@
         <v>27</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>28</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K19" s="7" t="s">
         <v>31</v>
@@ -2077,12 +2083,12 @@
         <v>26</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A20" s="29" t="s">
-        <v>226</v>
+      <c r="A20" s="20" t="s">
+        <v>224</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>12</v>
@@ -2097,19 +2103,19 @@
         <v>18</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K20" s="7" t="s">
         <v>31</v>
@@ -2118,12 +2124,12 @@
         <v>26</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A21" s="29" t="s">
-        <v>227</v>
+      <c r="A21" s="20" t="s">
+        <v>225</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>12</v>
@@ -2138,19 +2144,19 @@
         <v>29</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>30</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K21" s="7" t="s">
         <v>31</v>
@@ -2159,12 +2165,12 @@
         <v>26</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
-        <v>228</v>
+      <c r="A22" s="20" t="s">
+        <v>226</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>12</v>
@@ -2176,22 +2182,22 @@
         <v>16</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K22" s="7" t="s">
         <v>31</v>
@@ -2200,12 +2206,12 @@
         <v>26</v>
       </c>
       <c r="M22" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A23" s="29" t="s">
-        <v>229</v>
+      <c r="A23" s="20" t="s">
+        <v>227</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>12</v>
@@ -2217,22 +2223,22 @@
         <v>16</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F23" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="H23" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="G23" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>153</v>
-      </c>
       <c r="I23" s="4" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K23" s="7" t="s">
         <v>31</v>
@@ -2241,12 +2247,12 @@
         <v>26</v>
       </c>
       <c r="M23" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A24" s="28" t="s">
-        <v>230</v>
+      <c r="A24" s="19" t="s">
+        <v>228</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>12</v>
@@ -2259,19 +2265,19 @@
         <v>32</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K24" s="7" t="s">
         <v>33</v>
@@ -2280,12 +2286,12 @@
         <v>26</v>
       </c>
       <c r="M24" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A25" s="28" t="s">
-        <v>231</v>
+      <c r="A25" s="19" t="s">
+        <v>229</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>12</v>
@@ -2295,22 +2301,22 @@
       </c>
       <c r="D25" s="7"/>
       <c r="E25" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K25" s="7" t="s">
         <v>33</v>
@@ -2319,12 +2325,12 @@
         <v>26</v>
       </c>
       <c r="M25" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="105" x14ac:dyDescent="0.3">
-      <c r="A26" s="28" t="s">
-        <v>232</v>
+      <c r="A26" s="19" t="s">
+        <v>230</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>12</v>
@@ -2333,39 +2339,39 @@
         <v>15</v>
       </c>
       <c r="D26" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="E26" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="F26" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K26" s="7" t="s">
         <v>35</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="G26" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="H26" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="J26" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="K26" s="7" t="s">
-        <v>36</v>
       </c>
       <c r="L26" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M26" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A27" s="28" t="s">
-        <v>233</v>
+      <c r="A27" s="19" t="s">
+        <v>231</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>12</v>
@@ -2374,39 +2380,39 @@
         <v>15</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>39</v>
+        <v>248</v>
       </c>
       <c r="E27" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G27" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="F27" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="G27" s="7" t="s">
-        <v>38</v>
-      </c>
       <c r="H27" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L27" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M27" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="28" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A28" s="28" t="s">
-        <v>234</v>
+      <c r="A28" s="19" t="s">
+        <v>232</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>12</v>
@@ -2415,39 +2421,39 @@
         <v>15</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>39</v>
+        <v>250</v>
       </c>
       <c r="E28" s="9" t="s">
         <v>17</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K28" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L28" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M28" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="180" x14ac:dyDescent="0.3">
-      <c r="A29" s="28" t="s">
-        <v>235</v>
+      <c r="A29" s="19" t="s">
+        <v>233</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>12</v>
@@ -2456,39 +2462,39 @@
         <v>15</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>34</v>
+        <v>251</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K29" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L29" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M29" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A30" s="28" t="s">
-        <v>236</v>
+      <c r="A30" s="19" t="s">
+        <v>234</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>12</v>
@@ -2497,39 +2503,39 @@
         <v>15</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>42</v>
+        <v>249</v>
       </c>
       <c r="E30" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="G30" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="F30" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>43</v>
-      </c>
       <c r="H30" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L30" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A31" s="28" t="s">
-        <v>237</v>
+      <c r="A31" s="19" t="s">
+        <v>235</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>12</v>
@@ -2538,39 +2544,39 @@
         <v>15</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E31" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="H31" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="F31" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="H31" s="4" t="s">
-        <v>138</v>
-      </c>
       <c r="I31" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L31" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M31" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="32" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A32" s="28" t="s">
-        <v>238</v>
+      <c r="A32" s="19" t="s">
+        <v>236</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>12</v>
@@ -2579,39 +2585,39 @@
         <v>15</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E32" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="F32" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="F32" s="9" t="s">
+      <c r="G32" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="G32" s="7" t="s">
+      <c r="H32" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="H32" s="4" t="s">
-        <v>161</v>
-      </c>
       <c r="I32" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K32" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L32" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M32" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="33" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A33" s="28" t="s">
-        <v>239</v>
+      <c r="A33" s="19" t="s">
+        <v>237</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>12</v>
@@ -2620,39 +2626,39 @@
         <v>15</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E33" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="F33" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="F33" s="9" t="s">
+      <c r="G33" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="G33" s="7" t="s">
-        <v>160</v>
-      </c>
       <c r="H33" s="4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K33" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L33" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M33" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="34" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A34" s="28" t="s">
-        <v>240</v>
+      <c r="A34" s="19" t="s">
+        <v>238</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>12</v>
@@ -2661,39 +2667,39 @@
         <v>15</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K34" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L34" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M34" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="35" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A35" s="28" t="s">
-        <v>241</v>
+      <c r="A35" s="19" t="s">
+        <v>239</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>12</v>
@@ -2702,39 +2708,39 @@
         <v>15</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L35" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M35" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="36" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A36" s="28" t="s">
-        <v>242</v>
+      <c r="A36" s="19" t="s">
+        <v>240</v>
       </c>
       <c r="B36" s="7" t="s">
         <v>12</v>
@@ -2743,39 +2749,39 @@
         <v>15</v>
       </c>
       <c r="D36" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E36" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E36" s="9" t="s">
-        <v>46</v>
-      </c>
       <c r="F36" s="18" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K36" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L36" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M36" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="37" spans="1:13" ht="105" x14ac:dyDescent="0.3">
-      <c r="A37" s="28" t="s">
-        <v>243</v>
+      <c r="A37" s="19" t="s">
+        <v>241</v>
       </c>
       <c r="B37" s="7" t="s">
         <v>12</v>
@@ -2784,39 +2790,39 @@
         <v>15</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K37" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L37" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M37" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="38" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A38" s="28" t="s">
-        <v>244</v>
+      <c r="A38" s="19" t="s">
+        <v>242</v>
       </c>
       <c r="B38" s="7" t="s">
         <v>12</v>
@@ -2825,39 +2831,39 @@
         <v>15</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K38" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="L38" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M38" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="39" spans="1:13" ht="120" x14ac:dyDescent="0.3">
-      <c r="A39" s="28" t="s">
-        <v>245</v>
+      <c r="A39" s="19" t="s">
+        <v>243</v>
       </c>
       <c r="B39" s="7" t="s">
         <v>12</v>
@@ -2866,39 +2872,39 @@
         <v>15</v>
       </c>
       <c r="D39" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="J39" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K39" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="E39" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="F39" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="G39" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="H39" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="I39" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="J39" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="K39" s="7" t="s">
-        <v>51</v>
       </c>
       <c r="L39" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M39" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="40" spans="1:13" ht="135" x14ac:dyDescent="0.3">
-      <c r="A40" s="28" t="s">
-        <v>246</v>
+      <c r="A40" s="19" t="s">
+        <v>244</v>
       </c>
       <c r="B40" s="7" t="s">
         <v>12</v>
@@ -2907,39 +2913,39 @@
         <v>15</v>
       </c>
       <c r="D40" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="F40" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="J40" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K40" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="E40" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="G40" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="H40" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="I40" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="J40" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="K40" s="7" t="s">
-        <v>51</v>
       </c>
       <c r="L40" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M40" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="41" spans="1:13" ht="75" x14ac:dyDescent="0.3">
-      <c r="A41" s="28" t="s">
-        <v>247</v>
+      <c r="A41" s="19" t="s">
+        <v>245</v>
       </c>
       <c r="B41" s="7" t="s">
         <v>12</v>
@@ -2948,34 +2954,34 @@
         <v>15</v>
       </c>
       <c r="D41" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="J41" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K41" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="E41" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F41" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="G41" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="J41" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="K41" s="7" t="s">
-        <v>51</v>
       </c>
       <c r="L41" s="4" t="s">
         <v>26</v>
       </c>
       <c r="M41" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>